<commit_message>
Denetim raporuna 'Yeniden Üretilecekler' sekmesi eklendi
21 kıyafet parça sayfası (kategori B, hiç teslim edilmedi) ve iki yanlış
konulu ikonun (p3_agility, p5_scout) tam prompt metni tek bir sekmede -
Gemini'ye doğrudan yapıştırılabilir.

Claude-Session: https://claude.ai/code/session_01SmgLRHV2q6VtZPZSSuowT6
</commit_message>
<xml_diff>
--- a/docs/wayborne_gorsel_denetim.xlsx
+++ b/docs/wayborne_gorsel_denetim.xlsx
@@ -8,10 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Denetim" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ozet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Yeniden Üretilecekler" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ozet" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Denetim'!$A$1:$M$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Yeniden Üretilecekler'!$A$1:$H$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -126,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -172,6 +174,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8399,6 +8404,1035 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Gorsel / Item Adi</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Prompt Metni (Ingilizce - Gemini'ye yapistirilacak)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Cikti Dosya Adi</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Referans Gorsel Dosyasi</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>En-Boy Orani</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Neden yeniden isteniyor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>B-00</t>
+        </is>
+      </c>
+      <c r="B2" s="26" t="n">
+        <v>52000</v>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>body (skin layer)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: The bare body itself, as a SKIN LAYER. Paint every cell except "weapon": head (bald head, simple ear, neck, a plain profile face with only a small nose and brow line, no hair), torso, upper arm, forearm, hand (closed loosely, thumb forward), thigh, shin, foot (bare foot, sole on the red-dot line). Paint it in NEUTRAL LIGHT GREY tones only (#D8D8D8 base, #A8A8A8 shade, dark ink contour) — the game tints it with each character's skin colour.
+Cells: head, torso, upper_arm, forearm, hand, thigh, shin, foot.</t>
+        </is>
+      </c>
+      <c r="E2" s="26" t="inlineStr">
+        <is>
+          <t>body.png</t>
+        </is>
+      </c>
+      <c r="F2" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G2" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t>B-01</t>
+        </is>
+      </c>
+      <c r="B3" s="26" t="n">
+        <v>52101</v>
+      </c>
+      <c r="C3" s="26" t="inlineStr">
+        <is>
+          <t>hat_felt (Felt Cap)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: A soft felt cap in faded brown (#6B5238), the kind worn by nomads and drovers: rounded crown, a short upturned brim at the front, a stitched seam along the side. It sits on top of the head down to the ears; the face stays empty.
+Cells: head only.</t>
+        </is>
+      </c>
+      <c r="E3" s="26" t="inlineStr">
+        <is>
+          <t>hat_felt.png</t>
+        </is>
+      </c>
+      <c r="F3" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G3" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>B-02</t>
+        </is>
+      </c>
+      <c r="B4" s="26" t="n">
+        <v>52102</v>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>hat_hood (Travelling Hood)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: A grey-brown wool travelling hood (#4D4D57) pulled over the head, drawn slightly forward over the brow, falling to the neck and the top of the shoulders. The face opening stays empty. The hood's lower edge may spill a little into the top of the torso cell as a short shoulder cape.
+Cells: head (main), torso (only the short shoulder cape, top edge).</t>
+        </is>
+      </c>
+      <c r="E4" s="26" t="inlineStr">
+        <is>
+          <t>hat_hood.png</t>
+        </is>
+      </c>
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G4" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>B-03</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="n">
+        <v>52103</v>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>shirt_linen (Linen Shirt)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: A plain undyed linen shirt (#D1C7A8), loose and slightly creased, collarless with a short slit at the neck, long sleeves ending just above the wrist, hem tucked at the waist. Thin, soft fabric.
+Cells: torso, upper_arm, forearm.</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>shirt_linen.png</t>
+        </is>
+      </c>
+      <c r="F5" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G5" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>B-04</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="n">
+        <v>52104</v>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>shirt_dyed (Dyed Shirt)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: A woad-dyed blue linen shirt (#5C7594), faded unevenly from sun and washing, a narrow woven band along the collar and cuffs in pale gold (#DCB357). Long sleeves to the wrist, belted at the waist with a thin cord.
+Cells: torso, upper_arm, forearm.</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>shirt_dyed.png</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G6" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>B-05</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="n">
+        <v>52105</v>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>jacket_wool (Wool Coat)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: A heavy brown wool kaftan-style coat (#614733), wrapped across the chest and tied at the side, reaching mid-thigh, long sleeves slightly wider at the cuff, a darker felt trim along the front edge and hem. Worn patches at the elbows.
+Cells: torso (with the coat's skirt hanging below the hip), upper_arm, forearm, thigh (only the coat's skirt over the upper thigh).</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>jacket_wool.png</t>
+        </is>
+      </c>
+      <c r="F7" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G7" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>B-06</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="n">
+        <v>52106</v>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>jacket_leather (Leather Jerkin)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: A dark oiled leather jerkin (#4D3324), sleeveless body with short cap sleeves over the shoulder, laced up the front with leather thongs, scuffed and creased, a broad belt with a simple iron buckle.
+Cells: torso, upper_arm (cap sleeve only, top third).</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>jacket_leather.png</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G8" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>B-07</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="n">
+        <v>52107</v>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>gloves_leather (Leather Gloves)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: Brown work gloves of thick leather (#57402E) with a short flared cuff that covers the lower forearm, stitched seams on the back of the hand.
+Cells: hand, forearm (only the cuff, near the blue-dot end).</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>gloves_leather.png</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G9" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>B-08</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="n">
+        <v>52108</v>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>pants_wool (Wool Trousers)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: Dark grey-brown wool trousers (#47423D), loose at the thigh, wrapped tight below the knee with cloth puttee bands up the shin.
+Cells: thigh, shin.</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>pants_wool.png</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G10" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>B-09</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="n">
+        <v>52109</v>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>pants_canvas (Canvas Trousers)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: Light sand-coloured canvas trousers (#948A70), baggy in the Anatolian şalvar cut — full at the thigh, gathered at the ankle — dusty at the hem, a patched knee.
+Cells: thigh, shin.</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>pants_canvas.png</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G11" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>B-10</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="n">
+        <v>52110</v>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>shoes_boots (Riding Boots)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: Tall soft leather riding boots (#382920), reaching just below the knee, a slightly upturned toe, worn creases at the ankle, a thin sole. The sole must sit exactly on the red dot's horizontal line in the foot cell (that line is the ground).
+Cells: shin (boot shaft), foot.</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>shoes_boots.png</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G12" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>B-11</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="n">
+        <v>52111</v>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>shoes_sandals (Sandals)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: Simple leather sandals (#80664D): a flat sole with straps across the foot and two thin straps wrapping the lower ankle. The foot itself is NOT painted — only the sole and straps (the body layer shows through between the straps; leave those gaps empty).
+Cells: foot, shin (only the ankle straps at the lower end).</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>shoes_sandals.png</t>
+        </is>
+      </c>
+      <c r="F13" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G13" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>B-12</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="n">
+        <v>52112</v>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>armor_tier_1 (Leather Armor)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: Hardened boiled-leather armour: a thick quilted-and-leather cuirass covering chest and back to the hip, overlapping leather strips hanging over the upper thigh, small leather shoulder guards. Brown and dark tan (#5A3F2A / #7A5A3C), stitched, scuffed, matte.
+Cells: torso, upper_arm (shoulder guard, top third), thigh (hanging strips, top third).</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>armor_tier_1.png</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G14" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>B-13</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="n">
+        <v>52113</v>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>armor_tier_2 (Chain Shirt)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: A riveted iron mail shirt (cold steel #6F7A82, darker in the folds) reaching mid-thigh, with elbow-length mail sleeves, worn over a quilted under-coat whose padded edge shows at the neck and hem. The mail is shown as a fine ring texture, not individual shiny rings; dull, slightly rusty.
+Cells: torso, upper_arm, thigh (mail skirt, top half).</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>armor_tier_2.png</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G15" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>B-14</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="n">
+        <v>52114</v>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>armor_tier_3 (Plate Armor)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: Lamellar and plate armour of a veteran caravan guard: a chest of laced iron lamellae over mail, a rounded pauldron on the shoulder, a plate vambrace on the forearm, lamellar tassets over the thigh, a riveted iron gorget at the neck. Dull iron (#6F7A82) with dark leather lacing and a thin pale-gold (#DCB357) edge on the pauldron — worn, dented, never polished.
+Cells: torso, upper_arm, forearm, thigh.</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>armor_tier_3.png</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G16" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>B-15</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="n">
+        <v>52115</v>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>weapon_tier_1 (Caravan Sword)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: A plain iron arming sword for caravan guards: straight single-edged blade, simple cross guard, leather-wrapped grip, round iron pommel. Grey steel, a few nicks on the edge. Grip on the red dot, pommel just above it, blade pointing straight DOWN toward the blue dot and beyond.
+Cells: weapon only.</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>weapon_tier_1.png</t>
+        </is>
+      </c>
+      <c r="F17" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G17" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>B-16</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="n">
+        <v>52116</v>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>weapon_tier_2 (Master's Sword)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: A well-made curved sabre (kılıç): a slightly curved single-edged blade widening a little toward the tip, a short straight guard with downturned ends, a grip wrapped in dark leather, a brass (#DCB357, dulled) cap on the pommel. Grip on the red dot, blade pointing DOWN, the curve bending toward the right.
+Cells: weapon only.</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>weapon_tier_2.png</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G18" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>B-17</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="n">
+        <v>52117</v>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>weapon_tier_3 (Falcon Sword)</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: A fine old sabre of a master smith: a deeply curved blade with a subtle wavy forging pattern in the steel, a pale-gold (#DCB357) guard whose two ends are shaped like folded falcon wings, a grip bound in dark red cord (#A83029), a falcon-head pommel. Still worn and matte, not glowing. Grip on the red dot, blade pointing DOWN, curve bending toward the right.
+Cells: weapon only.</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>weapon_tier_3.png</t>
+        </is>
+      </c>
+      <c r="F19" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G19" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>B-18</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="n">
+        <v>52118</v>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>amulet_ward (Ward Charm)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: A small folded triangular cloth charm (muska) in faded red wool, stitched shut, hanging from a dark cord around the neck; the cord runs up toward the neck, the charm rests on the upper chest.
+Cells: torso only (upper chest, near the red dot).</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>amulet_ward.png</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G20" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>B-19</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="n">
+        <v>52119</v>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>amulet_wolf_fang (Wolf Fang Pendant)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: A single large yellowed wolf fang bound with a leather thong, hung on a braided cord around the neck, resting on the upper chest.
+Cells: torso only (upper chest).</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>amulet_wolf_fang.png</t>
+        </is>
+      </c>
+      <c r="F21" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G21" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>B-20</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="n">
+        <v>52120</v>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>amulet_courage (Courage Charm)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 2:3. Use the attached template.
+ITEM: A flat bronze disc pendant (dull #B08A4A), its face hammered with a simple radiating pattern (no letters, no religious sign), on a thin chain around the neck, resting on the upper chest.
+Cells: torso only (upper chest).</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>amulet_courage.png</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>part_sheet_template.png</t>
+        </is>
+      </c>
+      <c r="G22" s="26" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Bu teslimatta hiç gelmedi (kategori B - kıyafet parça sayfaları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>C-p3-agility</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="n">
+        <v>53102</v>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>a leaping hare mid-stride</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 1:1. ICON: a leaping hare mid-stride.</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>p3_agility.png</t>
+        </is>
+      </c>
+      <c r="F23" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G23" s="26" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>İlk teslimatta gelen dosya kendi dosya adıyla uyuşmuyordu (yumruk+halka, tavşan değil) - aynen aynı prompt'la tekrar iste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>C-p5-scout</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="n">
+        <v>53202</v>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>a hawk perched on a gloved fist</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Aspect ratio 1:1. ICON: a hawk perched on a gloved fist.</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>p5_scout.png</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="26" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>İlk teslimatta gelen dosya kendi dosya adıyla uyuşmuyordu (bir insan portresi, şahin değil) - aynen aynı prompt'la tekrar iste.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H24"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
İkonlar: stat/görev ailesi tek parşömen diskte (çeviklik, dayanıklılık, zekâ, sezgi, tellal), büyülü yüzüğün boncuğu mavi
</commit_message>
<xml_diff>
--- a/docs/wayborne_gorsel_denetim.xlsx
+++ b/docs/wayborne_gorsel_denetim.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2476,6 +2476,11 @@
           <t>Teslim edilen dosya p3_strength'in neredeyse kopyası (yumruk+halka). İstenen: sıçrayan tavşan. Şu an eski doğru ikon kullanılıyor.</t>
         </is>
       </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>ÇÖZÜLDÜ (2026-10-22): tavşan, ailenin parşömen diskine oturtuldu (tools/icon_discs.py).</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="32" t="inlineStr">
@@ -2523,6 +2528,11 @@
           <t>Teslim edilen bir insan portresi; ailenin geri kalanı hep nesne. İstenen: eldivenli yumruk üstünde şahin.</t>
         </is>
       </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>ÇÖZÜLDÜ (2026-10-22): gözcü portresi kalıyor - kullanıcı bu madalyonu örnek tasarım olarak gösterdi.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="32" t="inlineStr">
@@ -2570,6 +2580,11 @@
           <t>Kullanılabilir durumda; yalnızca mavi boncuk detayı eksik.</t>
         </is>
       </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>ÇÖZÜLDÜ (2026-10-22): kehribar boncuk maviye çevrildi (tools/icon_discs.py).</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="32" t="inlineStr">
@@ -2617,6 +2632,11 @@
           <t>Terazi geldi, defter+kalem istenmişti. Önceki turdan beri oyunda - değiştirmek de bırakmak da savunulabilir.</t>
         </is>
       </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>ÇÖZÜLDÜ (2026-10-22): terazi kalıyor, ailenin diskine oturtuldu.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="32" t="inlineStr">
@@ -2664,6 +2684,11 @@
           <t>Kırık mühür geldi, kırık asa istenmişti. Aynı durum.</t>
         </is>
       </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>ÇÖZÜLDÜ (2026-10-22): kırık mühür kalıyor - halefiyet sahnesinin çatlak mührüyle (G9b) aynı dil.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="31" t="inlineStr">
@@ -2803,6 +2828,13 @@
       <c r="I47" s="31" t="inlineStr">
         <is>
           <t>Prompt yolu bilerek terk edildi (7 tur). Model dosyası HENÜZ ELDE DEĞİL: main'e yüklenen zip 22 bayt, boş (GitHub web yükleyicisi 25 MB sınırlı). Bugünkü manken yer tutucu olarak çalışıyor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Ek (2026-10-22): p3_endurance gri kare, p3_perception kare karo, p5_crier çıplak çan geliyordu; üçü de ilk teslimatın/ikincinin temiz kaynağından aynı diske oturtuldu.</t>
         </is>
       </c>
     </row>

</xml_diff>